<commit_message>
docs(profiles): Loose seed profiles drop their volume floor to 0, matching the new default (CONTRACT-LIQUIDITY-DTE T2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BTHbXY65eM4aXdm97wSACP
</commit_message>
<xml_diff>
--- a/docs/search-profiles/Bamendjou_Options_Search_Profiles.xlsx
+++ b/docs/search-profiles/Bamendjou_Options_Search_Profiles.xlsx
@@ -684,7 +684,7 @@
         <v>0.2</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K2" s="4" t="n">
         <v>200</v>
@@ -752,7 +752,7 @@
         <v>0.2</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K3" s="4" t="n">
         <v>200</v>
@@ -956,7 +956,7 @@
         <v>0.3</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>75</v>
@@ -1024,7 +1024,7 @@
         <v>0.3</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>75</v>
@@ -1092,7 +1092,7 @@
         <v>0.2</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>200</v>
@@ -1160,7 +1160,7 @@
         <v>0.2</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K9" s="4" t="n">
         <v>200</v>
@@ -1364,7 +1364,7 @@
         <v>0.3</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>75</v>
@@ -1432,7 +1432,7 @@
         <v>0.3</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>75</v>
@@ -1500,7 +1500,7 @@
         <v>0.2</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K14" s="4" t="n">
         <v>200</v>
@@ -1568,7 +1568,7 @@
         <v>0.2</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>200</v>
@@ -1772,7 +1772,7 @@
         <v>0.3</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>75</v>
@@ -1840,7 +1840,7 @@
         <v>0.3</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>75</v>
@@ -1971,7 +1971,7 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">                 SemiAnnual_Restrictive keeps volume at the Baseline floor (50): a single ~200-DTE strike almost never trades</t>
+          <t xml:space="preserve">                 SemiAnnual_Restrictive keeps an explicit 50; the Baseline floor is now 0 (off): a single ~200-DTE strike almost never trades</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2013,7 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Min Volume                Hard-reject floor -- dropped if volume is below this</t>
+          <t xml:space="preserve">  Min Volume                Optional hard floor; 0 = off -- dropped if volume is below this</t>
         </is>
       </c>
     </row>
@@ -2041,14 +2041,14 @@
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Preferred Min Volume       Soft-rank threshold -- below this, scored down and flagged 'low_volume'.</t>
+          <t xml:space="preserve">  Preferred Min Volume       Soft-rank threshold -- below this, scored down and flagged 'thin_liquidity' (volume and open interest together count as one soft miss).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Preferred Min OI           Soft-rank threshold -- below this, scored down and flagged 'low_open_interest'.</t>
+          <t xml:space="preserve">  Preferred Min OI           Soft-rank threshold -- below this, scored down and flagged 'thin_liquidity' (volume and open interest together count as one soft miss).</t>
         </is>
       </c>
     </row>

</xml_diff>